<commit_message>
Modify File and Product For Bulk Cash Payment Command Request
</commit_message>
<xml_diff>
--- a/CBS.FrontDesk.UI/AppFiles/BulkOperation/BulkOperationFileUpload.xlsx
+++ b/CBS.FrontDesk.UI/AppFiles/BulkOperation/BulkOperationFileUpload.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BORIS\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BORIS\source\repos\CBS.FrontDesk.UI\CBS.FrontDesk.UI\AppFiles\BulkOperation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{000C0978-B5AB-41C2-9A3E-82521A1FBE28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F12B52F5-54A9-4E52-A3D4-F8AC7735FEE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6EB23830-41F9-440D-B3CF-7AD30EBE9D42}"/>
   </bookViews>
@@ -90,18 +90,6 @@
     <t>Account Type</t>
   </si>
   <si>
-    <t>Savings</t>
-  </si>
-  <si>
-    <t>Deposite</t>
-  </si>
-  <si>
-    <t>Preference Share</t>
-  </si>
-  <si>
-    <t>Member Share</t>
-  </si>
-  <si>
     <t>John Smith</t>
   </si>
   <si>
@@ -109,6 +97,18 @@
   </si>
   <si>
     <t>003</t>
+  </si>
+  <si>
+    <t>Deposit</t>
+  </si>
+  <si>
+    <t>PreferenceShare</t>
+  </si>
+  <si>
+    <t>MemberShare</t>
+  </si>
+  <si>
+    <t>Saving</t>
   </si>
 </sst>
 </file>
@@ -284,6 +284,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -294,9 +297,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -635,40 +635,40 @@
         <v>1</v>
       </c>
       <c r="B2" s="1"/>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="12"/>
+      <c r="D2" s="8"/>
     </row>
     <row r="3" spans="1:4" ht="15">
       <c r="A3" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B3" s="1"/>
-      <c r="C3" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" s="11"/>
+      <c r="C3" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="12"/>
     </row>
     <row r="4" spans="1:4" ht="15.6">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="2"/>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="8"/>
+      <c r="D4" s="9"/>
     </row>
     <row r="5" spans="1:4" ht="15.6">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="2"/>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="9"/>
+      <c r="D5" s="10"/>
     </row>
     <row r="6" spans="1:4" ht="17.399999999999999">
       <c r="A6" s="7" t="s">
@@ -697,10 +697,10 @@
         <v>1</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>25</v>
       </c>
       <c r="D8" s="3">
         <v>150</v>
@@ -711,7 +711,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>10</v>
@@ -725,7 +725,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>11</v>
@@ -739,7 +739,7 @@
         <v>4</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>12</v>
@@ -753,7 +753,7 @@
         <v>5</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>13</v>
@@ -767,7 +767,7 @@
         <v>6</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>14</v>
@@ -781,7 +781,7 @@
         <v>7</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>15</v>
@@ -795,7 +795,7 @@
         <v>8</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>16</v>
@@ -809,7 +809,7 @@
         <v>9</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>17</v>
@@ -823,7 +823,7 @@
         <v>10</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>18</v>

</xml_diff>